<commit_message>
Add cfb_analysis project to the page metadata files
</commit_message>
<xml_diff>
--- a/data/page_metadata.xlsx
+++ b/data/page_metadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cdpet\Documents\Post School Coursework\Portfolio Website\portfolio-website\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB044C40-1D12-4A81-88C4-06FA5903BB50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1F16E5-38D9-48D0-A015-FC9FF29A04F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{0F48850E-ADBC-4F08-8282-8BC2E517D1A7}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="125">
   <si>
     <t>python</t>
   </si>
@@ -69,9 +69,6 @@
     <t>Python</t>
   </si>
   <si>
-    <t>PCA, k-means clustering</t>
-  </si>
-  <si>
     <t>libraries_tools</t>
   </si>
   <si>
@@ -87,12 +84,6 @@
     <t>pandas, sklearn, imblearn</t>
   </si>
   <si>
-    <t>resampling, ensemble methods</t>
-  </si>
-  <si>
-    <t>database, web scraping, app</t>
-  </si>
-  <si>
     <t xml:space="preserve">pandas, splinter, bs4 (beautiful soup 4), bootstrap, mongodb, flask </t>
   </si>
   <si>
@@ -123,9 +114,6 @@
     <t>surf_weather</t>
   </si>
   <si>
-    <t>ETL</t>
-  </si>
-  <si>
     <t>pandas, sqlalchemy</t>
   </si>
   <si>
@@ -138,9 +126,6 @@
     <t>movies_etl</t>
   </si>
   <si>
-    <t>API</t>
-  </si>
-  <si>
     <t>https://github.com/cdpeters/weather-and-map-apis-python</t>
   </si>
   <si>
@@ -192,9 +177,6 @@
     <t>pandas, dash, ibis-framework, sqlite, tailwindcss</t>
   </si>
   <si>
-    <t>database, app</t>
-  </si>
-  <si>
     <t>nba_prediction</t>
   </si>
   <si>
@@ -204,9 +186,6 @@
     <t>About Me</t>
   </si>
   <si>
-    <t>linear regression, t-test, hypothesis testing, study design</t>
-  </si>
-  <si>
     <t>dplyr</t>
   </si>
   <si>
@@ -279,9 +258,6 @@
     <t>pandas, flask, flask-sqlalchemy, flask-caching, sqlalchemy, selectolax, selenium, beautifulsoup4, seaborn, python-dotenv, scikit-learn, ibis-framework, AWS, railway.app</t>
   </si>
   <si>
-    <t>database, web scraping, app, logistic regression, PCA, exploratory analysis</t>
-  </si>
-  <si>
     <t>https://nba-champion-analysis.up.railway.app/</t>
   </si>
   <si>
@@ -373,6 +349,57 @@
   </si>
   <si>
     <t>documentation, project setup, workflows</t>
+  </si>
+  <si>
+    <t>dataframe transformations, PCA, k-means clustering</t>
+  </si>
+  <si>
+    <t>dataframe transformations, resampling, ensemble methods</t>
+  </si>
+  <si>
+    <t>dataframe transformations, database, web scraping, app</t>
+  </si>
+  <si>
+    <t>dataframe transformations, database</t>
+  </si>
+  <si>
+    <t>dataframe transformations, ETL</t>
+  </si>
+  <si>
+    <t>dataframe transformations, API</t>
+  </si>
+  <si>
+    <t>dataframe transformations, database, app</t>
+  </si>
+  <si>
+    <t>dataframe transformations</t>
+  </si>
+  <si>
+    <t>dataframe transformations, database, web scraping, app, logistic regression, PCA, exploratory analysis</t>
+  </si>
+  <si>
+    <t>dataframe transformations, linear regression, t-test, hypothesis testing, study design</t>
+  </si>
+  <si>
+    <t>cfb_analysis</t>
+  </si>
+  <si>
+    <t>CFB 25 Analysis</t>
+  </si>
+  <si>
+    <t>https://github.com/cdpeters/cfb-analysis</t>
+  </si>
+  <si>
+    <t>polars, altair, marimo, httpx</t>
+  </si>
+  <si>
+    <t>dataframe transformations, exploratory analysis, app</t>
+  </si>
+  <si>
+    <t>https://cdpeters.github.io/cfb-analysis/</t>
+  </si>
+  <si>
+    <t>CFB 25 Roster Analysis</t>
   </si>
 </sst>
 </file>
@@ -773,7 +800,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C2C412C-6E97-4788-869B-F51667F527C3}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -809,7 +836,7 @@
         <v>11</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H1" s="6" t="s">
         <v>10</v>
@@ -818,18 +845,18 @@
         <v>7</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B2" s="7">
         <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -839,6 +866,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="7">
+        <f>$B2+1</f>
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -857,459 +885,518 @@
         <v>1</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="34.799999999999997" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4" s="7">
+        <f t="shared" ref="B4:B21" si="0">$B3+1</f>
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="34.799999999999997" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B5" s="7">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B6" s="7">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>27</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B7" s="7">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>32</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B8" s="7">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B9" s="7">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B10" s="7">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B11" s="7">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>55</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="52.2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="B12" s="7">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>65</v>
+        <v>118</v>
       </c>
       <c r="B13" s="7">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>63</v>
+        <v>119</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>62</v>
+        <v>120</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>60</v>
+        <v>13</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>121</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>59</v>
+        <v>122</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B14" s="7">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="7">
-        <v>12</v>
-      </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="E14" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="I14" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="H14" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="34.799999999999997" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="B15" s="7">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>77</v>
+        <v>56</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>76</v>
+        <v>55</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>27</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="B16" s="7">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>89</v>
+        <v>62</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>61</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>90</v>
+      <c r="G16" s="4" t="s">
+        <v>60</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>91</v>
+        <v>115</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="B17" s="7">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="B18" s="7">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="F18" s="1" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="B19" s="7">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="B20" s="7">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>113</v>
+        <v>80</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G20" s="1"/>
+        <v>13</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="H20" s="4" t="s">
-        <v>115</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B21" s="7">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" s="1"/>
+      <c r="H21" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1324,20 +1411,22 @@
     <hyperlink ref="E10" r:id="rId8" xr:uid="{08DF44EB-DC79-4D92-A240-4E05E17FBDF7}"/>
     <hyperlink ref="E11" r:id="rId9" xr:uid="{DFA5D084-673E-4D85-BBCF-AEC96AB4B5D1}"/>
     <hyperlink ref="E12" r:id="rId10" xr:uid="{3594118F-A025-4375-8B1A-478101EBBD1E}"/>
-    <hyperlink ref="E13" r:id="rId11" xr:uid="{C97D4B86-4F17-4BE5-8771-40E4B8A8781F}"/>
-    <hyperlink ref="E14" r:id="rId12" xr:uid="{D4592C7E-1F81-49BA-8CD3-AEC64D82E9B6}"/>
-    <hyperlink ref="I14" r:id="rId13" xr:uid="{9F657C65-7C4B-4A61-9A28-012A2D8E8603}"/>
-    <hyperlink ref="E15" r:id="rId14" xr:uid="{31227D6A-73B4-49CC-8654-EDFA7CEF3BA3}"/>
+    <hyperlink ref="E15" r:id="rId11" xr:uid="{C97D4B86-4F17-4BE5-8771-40E4B8A8781F}"/>
+    <hyperlink ref="E16" r:id="rId12" xr:uid="{D4592C7E-1F81-49BA-8CD3-AEC64D82E9B6}"/>
+    <hyperlink ref="I16" r:id="rId13" xr:uid="{9F657C65-7C4B-4A61-9A28-012A2D8E8603}"/>
+    <hyperlink ref="E14" r:id="rId14" xr:uid="{31227D6A-73B4-49CC-8654-EDFA7CEF3BA3}"/>
     <hyperlink ref="I12" r:id="rId15" xr:uid="{1B953180-0FFE-4C5F-864A-6BAAD97C1C06}"/>
-    <hyperlink ref="E16" r:id="rId16" xr:uid="{1C554EC0-F00A-43F4-8835-9026917B0DAA}"/>
+    <hyperlink ref="E20" r:id="rId16" xr:uid="{1C554EC0-F00A-43F4-8835-9026917B0DAA}"/>
     <hyperlink ref="E17" r:id="rId17" xr:uid="{5DC278CA-58BA-4869-993E-EFCED176BC66}"/>
     <hyperlink ref="E18" r:id="rId18" xr:uid="{76992F90-2A53-4B12-B9F8-0FE00BE22385}"/>
     <hyperlink ref="I18" r:id="rId19" xr:uid="{A0455F4C-62DE-4375-A61D-FCFC45FE70B4}"/>
     <hyperlink ref="E19" r:id="rId20" xr:uid="{3DA97EF0-4E20-4D79-AA49-98677FFD5404}"/>
     <hyperlink ref="I19" r:id="rId21" xr:uid="{AFC25449-4BF1-41AC-BA86-A7F8A4614DCE}"/>
-    <hyperlink ref="E20" r:id="rId22" xr:uid="{0B43302E-7669-49DC-BA1D-25CECB4B6EFB}"/>
+    <hyperlink ref="E21" r:id="rId22" xr:uid="{0B43302E-7669-49DC-BA1D-25CECB4B6EFB}"/>
+    <hyperlink ref="E13" r:id="rId23" xr:uid="{B9B52198-0FCF-4962-B764-6652E28CED63}"/>
+    <hyperlink ref="I13" r:id="rId24" xr:uid="{AC7B633F-BF88-49C1-822F-BB5B7C9DAD1C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId23"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Modify cfb-analysis project to use the new repo name 'cfb-25-analysis'
</commit_message>
<xml_diff>
--- a/data/page_metadata.xlsx
+++ b/data/page_metadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cdpet\Documents\Post School Coursework\Portfolio Website\portfolio-website\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1F16E5-38D9-48D0-A015-FC9FF29A04F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1274B0FF-798C-4FDA-A484-A8D4045A41FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{0F48850E-ADBC-4F08-8282-8BC2E517D1A7}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="124">
   <si>
     <t>python</t>
   </si>
@@ -381,25 +381,22 @@
     <t>dataframe transformations, linear regression, t-test, hypothesis testing, study design</t>
   </si>
   <si>
-    <t>cfb_analysis</t>
-  </si>
-  <si>
-    <t>CFB 25 Analysis</t>
-  </si>
-  <si>
-    <t>https://github.com/cdpeters/cfb-analysis</t>
-  </si>
-  <si>
     <t>polars, altair, marimo, httpx</t>
   </si>
   <si>
     <t>dataframe transformations, exploratory analysis, app</t>
   </si>
   <si>
-    <t>https://cdpeters.github.io/cfb-analysis/</t>
-  </si>
-  <si>
     <t>CFB 25 Roster Analysis</t>
+  </si>
+  <si>
+    <t>cfb_25_analysis</t>
+  </si>
+  <si>
+    <t>https://github.com/cdpeters/cfb-25-analysis</t>
+  </si>
+  <si>
+    <t>https://cdpeters.github.io/cfb-25-analysis/</t>
   </si>
 </sst>
 </file>
@@ -1139,7 +1136,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B13" s="7">
         <f t="shared" si="0"/>
@@ -1149,25 +1146,25 @@
         <v>0</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>123</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">

</xml_diff>